<commit_message>
changed questio status, add new question to QnA file on task 1
</commit_message>
<xml_diff>
--- a/Task 1/HV_QnA_Documen.xlsx
+++ b/Task 1/HV_QnA_Documen.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="21">
   <si>
     <t>No.</t>
   </si>
@@ -45,6 +45,9 @@
   </si>
   <si>
     <t>Phuc.pdd</t>
+  </si>
+  <si>
+    <t>Open</t>
   </si>
   <si>
     <t>Tính năng "Quên mật khẩu" sẽ hoạt động bằng cách nào ạ ? 
@@ -99,6 +102,9 @@
 Thay đổi mật khẩu (CHANGE PASSWORD)
 Lấy mật khẩu mới do quên mật khẩu (FORGOT PASSWORD) qua email"
 Theo Em hiểu thì NO_USER cũng nên có chức năng đăng nhập và quên mật khẩu phải không ạ ? trừ khi no user là người dùng chưa có tài khoản nhưng nhưng trong URD ghi là người dùng chưa đăng nhập</t>
+  </si>
+  <si>
+    <t>Em không thấy đề cập đến chức năng đăng xuất vậy nó không cần bao gồm trong srs phải không ạ ? hay nên được xem như chức năng nâng cao ạ ?</t>
   </si>
 </sst>
 </file>
@@ -475,7 +481,9 @@
       <c r="E2" s="5"/>
       <c r="F2" s="7"/>
       <c r="G2" s="8"/>
-      <c r="H2" s="5"/>
+      <c r="H2" s="5" t="s">
+        <v>11</v>
+      </c>
       <c r="I2" s="4"/>
       <c r="J2" s="4"/>
       <c r="K2" s="4"/>
@@ -503,7 +511,7 @@
         <v>8</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>10</v>
@@ -511,7 +519,9 @@
       <c r="E3" s="5"/>
       <c r="F3" s="7"/>
       <c r="G3" s="8"/>
-      <c r="H3" s="5"/>
+      <c r="H3" s="5" t="s">
+        <v>11</v>
+      </c>
       <c r="I3" s="4"/>
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
@@ -536,10 +546,10 @@
         <v>3.0</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>10</v>
@@ -547,7 +557,9 @@
       <c r="E4" s="5"/>
       <c r="F4" s="7"/>
       <c r="G4" s="8"/>
-      <c r="H4" s="5"/>
+      <c r="H4" s="5" t="s">
+        <v>11</v>
+      </c>
       <c r="I4" s="4"/>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
@@ -572,10 +584,10 @@
         <v>4.0</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D5" s="6" t="s">
         <v>10</v>
@@ -583,7 +595,9 @@
       <c r="E5" s="5"/>
       <c r="F5" s="7"/>
       <c r="G5" s="8"/>
-      <c r="H5" s="5"/>
+      <c r="H5" s="5" t="s">
+        <v>11</v>
+      </c>
       <c r="I5" s="4"/>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -608,10 +622,10 @@
         <v>5.0</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>10</v>
@@ -619,7 +633,9 @@
       <c r="E6" s="5"/>
       <c r="F6" s="7"/>
       <c r="G6" s="8"/>
-      <c r="H6" s="5"/>
+      <c r="H6" s="5" t="s">
+        <v>11</v>
+      </c>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -644,10 +660,10 @@
         <v>6.0</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>10</v>
@@ -655,7 +671,9 @@
       <c r="E7" s="5"/>
       <c r="F7" s="7"/>
       <c r="G7" s="8"/>
-      <c r="H7" s="5"/>
+      <c r="H7" s="5" t="s">
+        <v>11</v>
+      </c>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -679,15 +697,21 @@
       <c r="A8" s="5">
         <v>7.0</v>
       </c>
-      <c r="B8" s="6"/>
-      <c r="C8" s="6"/>
+      <c r="B8" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>20</v>
+      </c>
       <c r="D8" s="6" t="s">
         <v>10</v>
       </c>
       <c r="E8" s="5"/>
       <c r="F8" s="7"/>
       <c r="G8" s="8"/>
-      <c r="H8" s="5"/>
+      <c r="H8" s="5" t="s">
+        <v>11</v>
+      </c>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
       <c r="K8" s="4"/>

</xml_diff>